<commit_message>
feat: função que  ordena os produtos por volume de vendas do maior para o menor
</commit_message>
<xml_diff>
--- a/sales/sales.xlsx
+++ b/sales/sales.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -515,12 +515,35 @@
       <c r="E4" t="n">
         <v>484</v>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
+      <c r="F4" t="n">
+        <v>22</v>
       </c>
       <c r="G4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr"/>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>celular</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E5" t="n">
+        <v>2000</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>12/12/2025</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: Restaura salvamento no Excel removido na sale()
</commit_message>
<xml_diff>
--- a/sales/sales.xlsx
+++ b/sales/sales.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -544,6 +544,31 @@
         </is>
       </c>
       <c r="G5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr"/>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>teste de data</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>12/12/2021</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(xlsx): limpeza base de dados em planilha excel apontando para produtos eletrônicos
</commit_message>
<xml_diff>
--- a/sales/sales.xlsx
+++ b/sales/sales.xlsx
@@ -1,102 +1,37 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\55219\Documents\Isa - Documentos\Faculdade - UVA\4° Período - 2026.2\Análise de dados com Big Data\AV1\ccomp-4s-anbd-a4\sales\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7230"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="sales" sheetId="1" r:id="rId1"/>
+    <sheet name="sales" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="20">
-  <si>
-    <t>Produto</t>
-  </si>
-  <si>
-    <t>Preço</t>
-  </si>
-  <si>
-    <t>Quantidade</t>
-  </si>
-  <si>
-    <t>Valor</t>
-  </si>
-  <si>
-    <t>Data</t>
-  </si>
-  <si>
-    <t>id</t>
-  </si>
-  <si>
-    <t>3600.00</t>
-  </si>
-  <si>
-    <t>1800.00</t>
-  </si>
-  <si>
-    <t>Smartphone Galaxy</t>
-  </si>
-  <si>
-    <t>Fone Bluetooth</t>
-  </si>
-  <si>
-    <t>Mouse Gamer</t>
-  </si>
-  <si>
-    <t>Teclado Mecânico</t>
-  </si>
-  <si>
-    <t>Monitor 24 Full HD</t>
-  </si>
-  <si>
-    <t>950.00</t>
-  </si>
-  <si>
-    <t>1900.00</t>
-  </si>
-  <si>
-    <t>350.00</t>
-  </si>
-  <si>
-    <t>360.00</t>
-  </si>
-  <si>
-    <t>120.00</t>
-  </si>
-  <si>
-    <t>600.00</t>
-  </si>
-  <si>
-    <t>150.00</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+  </numFmts>
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -114,28 +49,82 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -423,138 +412,181 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="6.140625" customWidth="1"/>
-    <col min="2" max="2" width="18.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13" customWidth="1"/>
-    <col min="6" max="6" width="12.5703125" customWidth="1"/>
-  </cols>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Produto</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Preço</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Quantidade</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Valor</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Smartphone Galaxy</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>1800</v>
+      </c>
+      <c r="D2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E2" t="n">
+        <v>3600</v>
+      </c>
+      <c r="F2" s="1" t="n">
+        <v>46096</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Fone Bluetooth</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>150</v>
+      </c>
+      <c r="D3" t="n">
+        <v>4</v>
+      </c>
+      <c r="E3" t="n">
+        <v>600</v>
+      </c>
+      <c r="F3" s="1" t="n">
+        <v>46101</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Mouse Gamer</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>120</v>
+      </c>
+      <c r="D4" t="n">
+        <v>3</v>
+      </c>
+      <c r="E4" t="n">
+        <v>360</v>
+      </c>
+      <c r="F4" s="1" t="n">
+        <v>46117</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Teclado Mecânico</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>350</v>
+      </c>
+      <c r="D5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" t="n">
+        <v>350</v>
+      </c>
+      <c r="F5" s="1" t="n">
+        <v>46124</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
         <v>5</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="1" t="s">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Monitor 24 Full HD</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>950</v>
+      </c>
+      <c r="D6" t="n">
         <v>2</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="1">
-        <v>1</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" s="1">
+      <c r="E6" t="n">
+        <v>1900</v>
+      </c>
+      <c r="F6" s="1" t="n">
+        <v>46144</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Caixa de som JBL</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>3000</v>
+      </c>
+      <c r="D7" t="n">
         <v>2</v>
       </c>
-      <c r="E2" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F2" s="2">
-        <v>46096</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="1">
-        <v>2</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="D3" s="1">
-        <v>4</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="F3" s="2">
-        <v>46101</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="1">
-        <v>3</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="D4" s="1">
-        <v>3</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="F4" s="2">
-        <v>46117</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="1">
-        <v>4</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D5" s="1">
-        <v>1</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="F5" s="2">
-        <v>46124</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="1">
-        <v>5</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D6" s="1">
-        <v>2</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="F6" s="2">
-        <v>46144</v>
+      <c r="E7" t="n">
+        <v>6000</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>24/09/2026</t>
+        </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>